<commit_message>
ci(dev): publish dev build from 4271afa64bf6ab2a2ec4b567b98f6f2f23a9fd5e 4271afa64bf6ab2a2ec4b567b98f6f2f23a9fd5e
</commit_message>
<xml_diff>
--- a/dev/StructureDefinition-ph-core-medication.xlsx
+++ b/dev/StructureDefinition-ph-core-medication.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="248">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-25T03:26:10+00:00</t>
+    <t>2026-03-25T03:31:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -507,9 +507,6 @@
   </si>
   <si>
     <t>Depending on the context of use, the code that was actually selected by the user (prescriber, dispenser, etc.) will have the coding.userSelected set to true.  As described in the coding datatype: "A coding may be marked as a "userSelected" if a user selected the particular coded value in a user interface (e.g. the user selects an item in a pick-list). If a user selected coding exists, it is the preferred choice for performing translations etc. Other codes can only be literal translations to alternative code systems, or codes at a lower level of granularity (e.g. a generic code for a vendor-specific primary one).</t>
-  </si>
-  <si>
-    <t>extensible</t>
   </si>
   <si>
     <t>http://doh.gov.ph/fhir/ph-core/ValueSet/drugs-vs</t>
@@ -2469,11 +2466,11 @@
         <v>78</v>
       </c>
       <c r="X12" t="s" s="2">
-        <v>157</v>
+        <v>112</v>
       </c>
       <c r="Y12" s="2"/>
       <c r="Z12" t="s" s="2">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AA12" t="s" s="2">
         <v>78</v>
@@ -2506,24 +2503,24 @@
         <v>100</v>
       </c>
       <c r="AK12" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AL12" t="s" s="2">
         <v>159</v>
       </c>
-      <c r="AL12" t="s" s="2">
+      <c r="AM12" t="s" s="2">
         <v>160</v>
       </c>
-      <c r="AM12" t="s" s="2">
+      <c r="AN12" t="s" s="2">
         <v>161</v>
-      </c>
-      <c r="AN12" t="s" s="2">
-        <v>162</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2549,13 +2546,13 @@
         <v>108</v>
       </c>
       <c r="L13" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="M13" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="M13" t="s" s="2">
+      <c r="N13" t="s" s="2">
         <v>165</v>
-      </c>
-      <c r="N13" t="s" s="2">
-        <v>166</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2581,14 +2578,14 @@
         <v>78</v>
       </c>
       <c r="X13" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="Y13" t="s" s="2">
         <v>167</v>
       </c>
-      <c r="Y13" t="s" s="2">
+      <c r="Z13" t="s" s="2">
         <v>168</v>
       </c>
-      <c r="Z13" t="s" s="2">
-        <v>169</v>
-      </c>
       <c r="AA13" t="s" s="2">
         <v>78</v>
       </c>
@@ -2605,7 +2602,7 @@
         <v>78</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>79</v>
@@ -2623,7 +2620,7 @@
         <v>78</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AM13" t="s" s="2">
         <v>78</v>
@@ -2634,10 +2631,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2660,13 +2657,13 @@
         <v>89</v>
       </c>
       <c r="K14" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="L14" t="s" s="2">
         <v>172</v>
       </c>
-      <c r="L14" t="s" s="2">
+      <c r="M14" t="s" s="2">
         <v>173</v>
-      </c>
-      <c r="M14" t="s" s="2">
-        <v>174</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2717,7 +2714,7 @@
         <v>78</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>79</v>
@@ -2732,24 +2729,24 @@
         <v>100</v>
       </c>
       <c r="AK14" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="AL14" t="s" s="2">
         <v>175</v>
       </c>
-      <c r="AL14" t="s" s="2">
+      <c r="AM14" t="s" s="2">
         <v>176</v>
       </c>
-      <c r="AM14" t="s" s="2">
+      <c r="AN14" t="s" s="2">
         <v>177</v>
-      </c>
-      <c r="AN14" t="s" s="2">
-        <v>178</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2775,13 +2772,13 @@
         <v>153</v>
       </c>
       <c r="L15" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="M15" t="s" s="2">
         <v>180</v>
       </c>
-      <c r="M15" t="s" s="2">
+      <c r="N15" t="s" s="2">
         <v>181</v>
-      </c>
-      <c r="N15" t="s" s="2">
-        <v>182</v>
       </c>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
@@ -2807,14 +2804,14 @@
         <v>78</v>
       </c>
       <c r="X15" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="Y15" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="Y15" t="s" s="2">
+      <c r="Z15" t="s" s="2">
         <v>184</v>
       </c>
-      <c r="Z15" t="s" s="2">
-        <v>185</v>
-      </c>
       <c r="AA15" t="s" s="2">
         <v>78</v>
       </c>
@@ -2831,7 +2828,7 @@
         <v>78</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>79</v>
@@ -2846,24 +2843,24 @@
         <v>100</v>
       </c>
       <c r="AK15" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="AL15" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="AL15" t="s" s="2">
+      <c r="AM15" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN15" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN15" t="s" s="2">
-        <v>188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2886,13 +2883,13 @@
         <v>89</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="L16" t="s" s="2">
         <v>190</v>
       </c>
-      <c r="L16" t="s" s="2">
+      <c r="M16" t="s" s="2">
         <v>191</v>
-      </c>
-      <c r="M16" t="s" s="2">
-        <v>192</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2943,7 +2940,7 @@
         <v>78</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>79</v>
@@ -2961,7 +2958,7 @@
         <v>78</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AM16" t="s" s="2">
         <v>78</v>
@@ -2972,10 +2969,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2998,16 +2995,16 @@
         <v>78</v>
       </c>
       <c r="K17" t="s" s="2">
+        <v>194</v>
+      </c>
+      <c r="L17" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="L17" t="s" s="2">
+      <c r="M17" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="M17" t="s" s="2">
+      <c r="N17" t="s" s="2">
         <v>197</v>
-      </c>
-      <c r="N17" t="s" s="2">
-        <v>198</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3057,7 +3054,7 @@
         <v>78</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>79</v>
@@ -3075,7 +3072,7 @@
         <v>78</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AM17" t="s" s="2">
         <v>78</v>
@@ -3086,10 +3083,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3112,13 +3109,13 @@
         <v>78</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="L18" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="L18" t="s" s="2">
+      <c r="M18" t="s" s="2">
         <v>202</v>
-      </c>
-      <c r="M18" t="s" s="2">
-        <v>203</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3169,7 +3166,7 @@
         <v>78</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>79</v>
@@ -3187,7 +3184,7 @@
         <v>78</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AM18" t="s" s="2">
         <v>78</v>
@@ -3198,10 +3195,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3230,7 +3227,7 @@
         <v>135</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N19" t="s" s="2">
         <v>137</v>
@@ -3283,7 +3280,7 @@
         <v>78</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>79</v>
@@ -3301,7 +3298,7 @@
         <v>78</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>78</v>
@@ -3312,14 +3309,14 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -3341,10 +3338,10 @@
         <v>134</v>
       </c>
       <c r="L20" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="M20" t="s" s="2">
         <v>211</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>212</v>
       </c>
       <c r="N20" t="s" s="2">
         <v>137</v>
@@ -3399,7 +3396,7 @@
         <v>78</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -3428,10 +3425,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3454,17 +3451,17 @@
         <v>78</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>214</v>
+      </c>
+      <c r="L21" t="s" s="2">
         <v>215</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>216</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>217</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" t="s" s="2">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>78</v>
@@ -3513,7 +3510,7 @@
         <v>78</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>88</v>
@@ -3528,24 +3525,24 @@
         <v>100</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AL21" t="s" s="2">
+        <v>218</v>
+      </c>
+      <c r="AM21" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN21" t="s" s="2">
         <v>219</v>
-      </c>
-      <c r="AM21" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN21" t="s" s="2">
-        <v>220</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3568,17 +3565,17 @@
         <v>78</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="L22" t="s" s="2">
         <v>222</v>
       </c>
-      <c r="L22" t="s" s="2">
+      <c r="M22" t="s" s="2">
         <v>223</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>224</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" t="s" s="2">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>78</v>
@@ -3627,7 +3624,7 @@
         <v>78</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -3645,7 +3642,7 @@
         <v>78</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>78</v>
@@ -3656,10 +3653,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3682,13 +3679,13 @@
         <v>78</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L23" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="M23" t="s" s="2">
         <v>228</v>
-      </c>
-      <c r="M23" t="s" s="2">
-        <v>229</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3739,7 +3736,7 @@
         <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>79</v>
@@ -3754,24 +3751,24 @@
         <v>100</v>
       </c>
       <c r="AK23" t="s" s="2">
+        <v>229</v>
+      </c>
+      <c r="AL23" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="AM23" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN23" t="s" s="2">
         <v>230</v>
-      </c>
-      <c r="AL23" t="s" s="2">
-        <v>193</v>
-      </c>
-      <c r="AM23" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN23" t="s" s="2">
-        <v>231</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3794,13 +3791,13 @@
         <v>78</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="L24" t="s" s="2">
+        <v>232</v>
+      </c>
+      <c r="M24" t="s" s="2">
         <v>233</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>234</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3851,7 +3848,7 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -3866,10 +3863,10 @@
         <v>100</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AM24" t="s" s="2">
         <v>78</v>
@@ -3880,10 +3877,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3906,13 +3903,13 @@
         <v>78</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="L25" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="L25" t="s" s="2">
+      <c r="M25" t="s" s="2">
         <v>202</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>203</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3963,7 +3960,7 @@
         <v>78</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -3981,7 +3978,7 @@
         <v>78</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>78</v>
@@ -3992,10 +3989,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4024,7 +4021,7 @@
         <v>135</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N26" t="s" s="2">
         <v>137</v>
@@ -4077,7 +4074,7 @@
         <v>78</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>79</v>
@@ -4095,7 +4092,7 @@
         <v>78</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>78</v>
@@ -4106,14 +4103,14 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4135,10 +4132,10 @@
         <v>134</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>211</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>212</v>
       </c>
       <c r="N27" t="s" s="2">
         <v>137</v>
@@ -4193,7 +4190,7 @@
         <v>78</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
@@ -4222,10 +4219,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4248,13 +4245,13 @@
         <v>78</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L28" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="M28" t="s" s="2">
         <v>240</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>241</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4305,7 +4302,7 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>79</v>
@@ -4320,7 +4317,7 @@
         <v>100</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>150</v>
@@ -4329,15 +4326,15 @@
         <v>78</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4360,13 +4357,13 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="L29" t="s" s="2">
+      <c r="M29" t="s" s="2">
         <v>245</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>246</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4417,7 +4414,7 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -4432,16 +4429,16 @@
         <v>100</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AL29" t="s" s="2">
+        <v>246</v>
+      </c>
+      <c r="AM29" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN29" t="s" s="2">
         <v>247</v>
-      </c>
-      <c r="AM29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN29" t="s" s="2">
-        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>